<commit_message>
Update crypto tracker data
</commit_message>
<xml_diff>
--- a/ATR_Tracker_Dashboard.xlsx
+++ b/ATR_Tracker_Dashboard.xlsx
@@ -2194,9 +2194,6 @@
           <t>1w</t>
         </is>
       </c>
-      <c r="D47" t="n">
-        <v/>
-      </c>
       <c r="E47" t="n">
         <v>6.881703635229012</v>
       </c>
@@ -2209,9 +2206,6 @@
       <c r="H47" t="n">
         <v>0.7302432273183066</v>
       </c>
-      <c r="J47" t="n">
-        <v/>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2267,9 +2261,6 @@
           <t>1w</t>
         </is>
       </c>
-      <c r="D49" t="n">
-        <v/>
-      </c>
       <c r="E49" t="n">
         <v>9.318927986926848</v>
       </c>
@@ -2282,9 +2273,6 @@
       <c r="H49" t="n">
         <v>0.5283678823589186</v>
       </c>
-      <c r="J49" t="n">
-        <v/>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2340,9 +2328,6 @@
           <t>1w</t>
         </is>
       </c>
-      <c r="D51" t="n">
-        <v/>
-      </c>
       <c r="E51" t="n">
         <v>10.0396551035204</v>
       </c>
@@ -2352,12 +2337,6 @@
       <c r="G51" t="n">
         <v>91.73694150948708</v>
       </c>
-      <c r="H51" t="n">
-        <v/>
-      </c>
-      <c r="J51" t="n">
-        <v/>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2413,9 +2392,6 @@
           <t>1w</t>
         </is>
       </c>
-      <c r="D53" t="n">
-        <v/>
-      </c>
       <c r="E53" t="n">
         <v>9.400787352855257</v>
       </c>
@@ -2425,12 +2401,6 @@
       <c r="G53" t="n">
         <v>97.68451508929084</v>
       </c>
-      <c r="H53" t="n">
-        <v/>
-      </c>
-      <c r="J53" t="n">
-        <v/>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2486,9 +2456,6 @@
           <t>1w</t>
         </is>
       </c>
-      <c r="D55" t="n">
-        <v/>
-      </c>
       <c r="E55" t="n">
         <v>8.667091027090382</v>
       </c>
@@ -2498,12 +2465,6 @@
       <c r="G55" t="n">
         <v>88.39881348364079</v>
       </c>
-      <c r="H55" t="n">
-        <v/>
-      </c>
-      <c r="J55" t="n">
-        <v/>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2570,9 +2531,6 @@
       </c>
       <c r="G57" t="n">
         <v>60.19344326541734</v>
-      </c>
-      <c r="H57" t="n">
-        <v/>
       </c>
       <c r="I57" t="n">
         <v>0.7282196589159247</v>

</xml_diff>